<commit_message>
Improve catering workflows, tenant login and role permissions
</commit_message>
<xml_diff>
--- a/public/samples/employees-import-example.xlsx
+++ b/public/samples/employees-import-example.xlsx
@@ -14,8 +14,34 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="T1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <b val="false"/>
+            <i val="false"/>
+            <strike val="false"/>
+            <color rgb="FF000000"/>
+            <sz val="11"/>
+            <u val="none"/>
+          </rPr>
+          <t xml:space="preserve">1 = fikcyjny PESEL, 0 = prawdziwy. Puste pole zachowuje dotychczasowe oznaczenie pracownika. PESEL, telefon i e-mail są wymagane; nazwisko i adres są opcjonalne.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="20">
   <si>
     <t>firstName</t>
   </si>
@@ -72,6 +98,9 @@
   </si>
   <si>
     <t>active</t>
+  </si>
+  <si>
+    <t>isPeselFake</t>
   </si>
 </sst>
 </file>
@@ -441,31 +470,32 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:T1"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="13.997" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="9.283" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="9.283" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="9.283" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="8.141" bestFit="true" customWidth="true" style="0"/>
-    <col min="9" max="9" width="11.569" bestFit="true" customWidth="true" style="0"/>
-    <col min="10" max="10" width="19.852" bestFit="true" customWidth="true" style="0"/>
-    <col min="11" max="11" width="19.852" bestFit="true" customWidth="true" style="0"/>
-    <col min="12" max="12" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="13" max="13" width="20.995" bestFit="true" customWidth="true" style="0"/>
-    <col min="14" max="14" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="15" max="15" width="25.708" bestFit="true" customWidth="true" style="0"/>
-    <col min="16" max="16" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="17" max="17" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="18" max="18" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="19" max="19" width="10.426" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="13.997" customWidth="true" style="0"/>
+    <col min="2" max="2" width="12.854" customWidth="true" style="0"/>
+    <col min="3" max="3" width="9.283" customWidth="true" style="0"/>
+    <col min="4" max="4" width="9.283" customWidth="true" style="0"/>
+    <col min="5" max="5" width="9.283" customWidth="true" style="0"/>
+    <col min="6" max="6" width="10.426" customWidth="true" style="0"/>
+    <col min="7" max="7" width="12.854" customWidth="true" style="0"/>
+    <col min="8" max="8" width="8.141" customWidth="true" style="0"/>
+    <col min="9" max="9" width="11.569" customWidth="true" style="0"/>
+    <col min="10" max="10" width="19.852" customWidth="true" style="0"/>
+    <col min="11" max="11" width="19.852" customWidth="true" style="0"/>
+    <col min="12" max="12" width="17.567" customWidth="true" style="0"/>
+    <col min="13" max="13" width="20.995" customWidth="true" style="0"/>
+    <col min="14" max="14" width="12.854" customWidth="true" style="0"/>
+    <col min="15" max="15" width="25.708" customWidth="true" style="0"/>
+    <col min="16" max="16" width="17.567" customWidth="true" style="0"/>
+    <col min="17" max="17" width="17.567" customWidth="true" style="0"/>
+    <col min="18" max="18" width="17.567" customWidth="true" style="0"/>
+    <col min="19" max="19" width="10.426" customWidth="true" style="0"/>
+    <col min="20" max="20" width="13.997" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -522,11 +552,15 @@
       </c>
       <c r="S1" s="2" t="s">
         <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <legacyDrawing r:id="rId_comments_vml1"/>
 </worksheet>
 </file>
</xml_diff>